<commit_message>
updated to N8R8 esp32 version
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget_MP.xlsx
+++ b/docs/05-Power-Budget/PowerBudget_MP.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="59">
   <si>
     <t>Power Budget - Mihir Patel</t>
   </si>
@@ -91,7 +91,7 @@
     <t>ESP32-S3-Wi-Fi Module</t>
   </si>
   <si>
-    <t>ESP32-S3-WROOM-1-N4</t>
+    <t>ESP32-S3-WROOM-1-N8R8</t>
   </si>
   <si>
     <t>3.3V</t>
@@ -100,10 +100,10 @@
     <t>mA</t>
   </si>
   <si>
-    <t>Camera moduel (OV2640)</t>
+    <t>Camera module (OV5640)</t>
   </si>
   <si>
-    <t>OV2640</t>
+    <t>OV5640</t>
   </si>
   <si>
     <t>Debug LEDs (SMD 0805)</t>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve"> +3.3V Power Rail</t>
+  </si>
+  <si>
+    <t>Camera moduel (OV5640)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal </t>
@@ -838,7 +841,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="26.11"/>
     <col customWidth="1" min="2" max="2" width="30.67"/>
-    <col customWidth="1" min="3" max="3" width="19.89"/>
+    <col customWidth="1" min="3" max="3" width="20.67"/>
     <col customWidth="1" min="4" max="4" width="11.44"/>
     <col customWidth="1" min="5" max="5" width="6.89"/>
     <col customWidth="1" min="6" max="6" width="12.33"/>
@@ -1505,7 +1508,7 @@
     <row r="19" ht="15.0" customHeight="1">
       <c r="A19" s="16"/>
       <c r="B19" s="17" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>23</v>
@@ -1715,7 +1718,7 @@
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="16"/>
       <c r="B24" s="28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G24" s="27">
         <f>SUM(G18:G23)</f>
@@ -1746,7 +1749,7 @@
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="16"/>
       <c r="B25" s="29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G25" s="30">
         <v>0.25</v>
@@ -1774,7 +1777,7 @@
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="16"/>
       <c r="B26" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G26" s="27">
         <f>G24*(1+G25)</f>
@@ -1832,16 +1835,16 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D28" s="35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E28" s="33">
         <v>1.0</v>
@@ -1878,7 +1881,7 @@
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="16"/>
       <c r="B29" s="37" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G29" s="38">
         <f>G28-G26</f>
@@ -1936,7 +1939,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
@@ -1994,7 +1997,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="46" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>11</v>
@@ -2038,16 +2041,16 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="47" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B34" s="47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E34" s="33">
         <v>1.0</v>
@@ -2111,7 +2114,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -2141,7 +2144,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>11</v>
@@ -2153,7 +2156,7 @@
         <v>13</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>15</v>
@@ -2185,19 +2188,19 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="50" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B38" s="51" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F38" s="52">
         <v>2500.0</v>
@@ -2257,7 +2260,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="59" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B40" s="56"/>
       <c r="C40" s="56"/>
@@ -2316,13 +2319,13 @@
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="60"/>
       <c r="B42" s="36" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D42" s="35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E42" s="33">
         <v>1.0</v>
@@ -2359,7 +2362,7 @@
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="55"/>
       <c r="B43" s="37" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G43" s="38">
         <f>G38-SUM(G40:G42)</f>
@@ -2445,7 +2448,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="65" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B46" s="66"/>
       <c r="C46" s="66"/>
@@ -2475,7 +2478,7 @@
     </row>
     <row r="47" ht="26.25" customHeight="1">
       <c r="A47" s="69" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
@@ -28014,9 +28017,17 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <printOptions/>
-  <pageMargins bottom="0.0" footer="0.0" header="0.0" left="0.0" right="0.0" top="0.0"/>
-  <pageSetup orientation="landscape"/>
+  <printOptions gridLines="1" horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.25" right="0.25" top="0.75"/>
+  <pageSetup paperSize="9" orientation="landscape"/>
+  <rowBreaks count="2" manualBreakCount="2">
+    <brk man="1"/>
+    <brk id="52" man="1"/>
+  </rowBreaks>
+  <colBreaks count="2" manualBreakCount="2">
+    <brk man="1"/>
+    <brk id="8" man="1"/>
+  </colBreaks>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated power budget and microcontroller section
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget_MP.xlsx
+++ b/docs/05-Power-Budget/PowerBudget_MP.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="64">
   <si>
     <t>Power Budget - Mihir Patel</t>
   </si>
@@ -206,6 +206,21 @@
     <t>Total Remaining Current Available on External Power Source 1</t>
   </si>
   <si>
+    <t>External Power Source 2</t>
+  </si>
+  <si>
+    <t>Power Source 2 Selection</t>
+  </si>
+  <si>
+    <t>Battery (12V) - Raunak's shared power</t>
+  </si>
+  <si>
+    <t>B09ZTKTLGW</t>
+  </si>
+  <si>
+    <t>12V</t>
+  </si>
+  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -293,7 +308,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border/>
     <border>
       <left style="thin">
@@ -411,12 +426,33 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <bottom style="thin">
+      <top style="thin">
         <color rgb="FF000000"/>
-      </bottom>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
     </border>
     <border>
       <right style="thin">
@@ -447,7 +483,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="79">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -550,13 +586,36 @@
     </xf>
     <xf borderId="11" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="12" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="13" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="13" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="14" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="15" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="10" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -574,7 +633,7 @@
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -586,7 +645,7 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="17" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -594,17 +653,19 @@
     <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="5" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="15" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="16" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="17" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="18" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="18" fillId="3" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="19" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="20" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="21" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1999,25 +2060,25 @@
       <c r="A33" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="D33" s="14" t="s">
+      <c r="D33" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="E33" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="F33" s="14" t="s">
+      <c r="F33" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="G33" s="26" t="s">
+      <c r="G33" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="H33" s="26" t="s">
+      <c r="H33" s="48" t="s">
         <v>17</v>
       </c>
       <c r="I33" s="2"/>
@@ -2040,29 +2101,29 @@
       <c r="Z33" s="2"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="47" t="s">
+      <c r="A34" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="B34" s="47" t="s">
+      <c r="B34" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="D34" s="35" t="s">
+      <c r="D34" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="E34" s="33">
+      <c r="E34" s="52">
         <v>1.0</v>
       </c>
-      <c r="F34" s="36">
+      <c r="F34" s="53">
         <v>2000.0</v>
       </c>
-      <c r="G34" s="27">
+      <c r="G34" s="54">
         <f>E34*F34</f>
         <v>2000</v>
       </c>
-      <c r="H34" s="27" t="s">
+      <c r="H34" s="54" t="s">
         <v>21</v>
       </c>
       <c r="I34" s="2"/>
@@ -2085,14 +2146,14 @@
       <c r="Z34" s="2"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="2"/>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
+      <c r="A35" s="55"/>
+      <c r="B35" s="56"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="56"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
@@ -2113,16 +2174,16 @@
       <c r="Z35" s="2"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="12"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="44"/>
+      <c r="F36" s="44"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="45"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
@@ -2155,7 +2216,7 @@
       <c r="D37" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="E37" s="49" t="s">
+      <c r="E37" s="58" t="s">
         <v>48</v>
       </c>
       <c r="F37" s="14" t="s">
@@ -2187,10 +2248,10 @@
       <c r="Z37" s="2"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="B38" s="51" t="s">
+      <c r="B38" s="60" t="s">
         <v>50</v>
       </c>
       <c r="C38" s="35" t="s">
@@ -2202,13 +2263,13 @@
       <c r="E38" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="F38" s="52">
+      <c r="F38" s="61">
         <v>2500.0</v>
       </c>
-      <c r="G38" s="53">
+      <c r="G38" s="62">
         <v>2500.0</v>
       </c>
-      <c r="H38" s="54" t="s">
+      <c r="H38" s="63" t="s">
         <v>21</v>
       </c>
       <c r="I38" s="2"/>
@@ -2231,14 +2292,14 @@
       <c r="Z38" s="2"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="55"/>
-      <c r="B39" s="56"/>
-      <c r="C39" s="56"/>
+      <c r="A39" s="64"/>
+      <c r="B39" s="65"/>
+      <c r="C39" s="65"/>
       <c r="D39" s="33"/>
       <c r="E39" s="33"/>
-      <c r="F39" s="57"/>
+      <c r="F39" s="66"/>
       <c r="G39" s="38"/>
-      <c r="H39" s="58"/>
+      <c r="H39" s="67"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
@@ -2259,14 +2320,14 @@
       <c r="Z39" s="2"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="59" t="s">
+      <c r="A40" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="56"/>
-      <c r="C40" s="56"/>
+      <c r="B40" s="65"/>
+      <c r="C40" s="65"/>
       <c r="D40" s="33"/>
       <c r="E40" s="33"/>
-      <c r="F40" s="57"/>
+      <c r="F40" s="66"/>
       <c r="G40" s="38"/>
       <c r="H40" s="27"/>
       <c r="I40" s="2"/>
@@ -2289,12 +2350,12 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="60"/>
-      <c r="B41" s="56"/>
-      <c r="C41" s="56"/>
+      <c r="A41" s="69"/>
+      <c r="B41" s="65"/>
+      <c r="C41" s="65"/>
       <c r="D41" s="33"/>
       <c r="E41" s="33"/>
-      <c r="F41" s="57"/>
+      <c r="F41" s="66"/>
       <c r="G41" s="38"/>
       <c r="H41" s="27"/>
       <c r="I41" s="2"/>
@@ -2317,7 +2378,7 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="60"/>
+      <c r="A42" s="69"/>
       <c r="B42" s="36" t="s">
         <v>55</v>
       </c>
@@ -2360,7 +2421,7 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="55"/>
+      <c r="A43" s="64"/>
       <c r="B43" s="37" t="s">
         <v>56</v>
       </c>
@@ -2368,7 +2429,7 @@
         <f>G38-SUM(G40:G42)</f>
         <v>500</v>
       </c>
-      <c r="H43" s="54" t="s">
+      <c r="H43" s="63" t="s">
         <v>21</v>
       </c>
       <c r="I43" s="2"/>
@@ -2391,14 +2452,14 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="55"/>
+      <c r="A44" s="64"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
-      <c r="G44" s="61"/>
-      <c r="H44" s="62"/>
+      <c r="G44" s="70"/>
+      <c r="H44" s="71"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -2419,14 +2480,30 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="41"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="33"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="64"/>
+      <c r="A45" s="72" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" s="58" t="s">
+        <v>48</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="G45" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" s="26" t="s">
+        <v>17</v>
+      </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
@@ -2447,16 +2524,30 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46" ht="15.0" customHeight="1">
-      <c r="A46" s="65" t="s">
-        <v>57</v>
+      <c r="A46" s="73" t="s">
+        <v>58</v>
       </c>
-      <c r="B46" s="66"/>
-      <c r="C46" s="66"/>
-      <c r="D46" s="66"/>
-      <c r="E46" s="66"/>
-      <c r="F46" s="67"/>
-      <c r="G46" s="68"/>
-      <c r="H46" s="68"/>
+      <c r="B46" s="60" t="s">
+        <v>59</v>
+      </c>
+      <c r="C46" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="E46" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="F46" s="61">
+        <v>7000.0</v>
+      </c>
+      <c r="G46" s="62">
+        <v>7000.0</v>
+      </c>
+      <c r="H46" s="63" t="s">
+        <v>21</v>
+      </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -2476,10 +2567,15 @@
       <c r="Y46" s="2"/>
       <c r="Z46" s="2"/>
     </row>
-    <row r="47" ht="26.25" customHeight="1">
-      <c r="A47" s="69" t="s">
-        <v>58</v>
-      </c>
+    <row r="47" ht="15.0" customHeight="1">
+      <c r="A47" s="64"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="66"/>
+      <c r="G47" s="38"/>
+      <c r="H47" s="67"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
@@ -2499,7 +2595,17 @@
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
     </row>
-    <row r="48" ht="36.0" customHeight="1">
+    <row r="48" ht="15.0" customHeight="1">
+      <c r="A48" s="68" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="65"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="33"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="27"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -2519,7 +2625,15 @@
       <c r="Y48" s="2"/>
       <c r="Z48" s="2"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="15.0" customHeight="1">
+      <c r="A49" s="69"/>
+      <c r="B49" s="65"/>
+      <c r="C49" s="65"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="66"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="27"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
@@ -2539,7 +2653,30 @@
       <c r="Y49" s="2"/>
       <c r="Z49" s="2"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="15.0" customHeight="1">
+      <c r="A50" s="69"/>
+      <c r="B50" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D50" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="E50" s="33">
+        <v>1.0</v>
+      </c>
+      <c r="F50" s="36">
+        <v>2000.0</v>
+      </c>
+      <c r="G50" s="27">
+        <f>E50*F50</f>
+        <v>2000</v>
+      </c>
+      <c r="H50" s="27" t="s">
+        <v>21</v>
+      </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
@@ -2559,7 +2696,18 @@
       <c r="Y50" s="2"/>
       <c r="Z50" s="2"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="15.0" customHeight="1">
+      <c r="A51" s="64"/>
+      <c r="B51" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="G51" s="38">
+        <f>G46-SUM(G48:G50)</f>
+        <v>5000</v>
+      </c>
+      <c r="H51" s="63" t="s">
+        <v>21</v>
+      </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
@@ -2579,7 +2727,17 @@
       <c r="Y51" s="2"/>
       <c r="Z51" s="2"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="15.0" customHeight="1">
+      <c r="A52" s="74" t="s">
+        <v>62</v>
+      </c>
+      <c r="B52" s="75"/>
+      <c r="C52" s="75"/>
+      <c r="D52" s="75"/>
+      <c r="E52" s="75"/>
+      <c r="F52" s="76"/>
+      <c r="G52" s="77"/>
+      <c r="H52" s="77"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
@@ -2599,15 +2757,10 @@
       <c r="Y52" s="2"/>
       <c r="Z52" s="2"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
+    <row r="53" ht="26.25" customHeight="1">
+      <c r="A53" s="78" t="s">
+        <v>63</v>
+      </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -2627,15 +2780,7 @@
       <c r="Y53" s="2"/>
       <c r="Z53" s="2"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
+    <row r="54" ht="36.0" customHeight="1">
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -2656,14 +2801,6 @@
       <c r="Z54" s="2"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
@@ -2684,14 +2821,6 @@
       <c r="Z55" s="2"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -2712,14 +2841,6 @@
       <c r="Z56" s="2"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
@@ -2740,14 +2861,6 @@
       <c r="Z57" s="2"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
@@ -27995,15 +28108,176 @@
       <c r="Y959" s="2"/>
       <c r="Z959" s="2"/>
     </row>
+    <row r="960" ht="15.75" customHeight="1">
+      <c r="A960" s="2"/>
+      <c r="B960" s="2"/>
+      <c r="C960" s="2"/>
+      <c r="D960" s="2"/>
+      <c r="E960" s="2"/>
+      <c r="F960" s="2"/>
+      <c r="G960" s="2"/>
+      <c r="H960" s="2"/>
+      <c r="I960" s="2"/>
+      <c r="J960" s="2"/>
+      <c r="K960" s="2"/>
+      <c r="L960" s="2"/>
+      <c r="M960" s="2"/>
+      <c r="N960" s="2"/>
+      <c r="O960" s="2"/>
+      <c r="P960" s="2"/>
+      <c r="Q960" s="2"/>
+      <c r="R960" s="2"/>
+      <c r="S960" s="2"/>
+      <c r="T960" s="2"/>
+      <c r="U960" s="2"/>
+      <c r="V960" s="2"/>
+      <c r="W960" s="2"/>
+      <c r="X960" s="2"/>
+      <c r="Y960" s="2"/>
+      <c r="Z960" s="2"/>
+    </row>
+    <row r="961" ht="15.75" customHeight="1">
+      <c r="A961" s="2"/>
+      <c r="B961" s="2"/>
+      <c r="C961" s="2"/>
+      <c r="D961" s="2"/>
+      <c r="E961" s="2"/>
+      <c r="F961" s="2"/>
+      <c r="G961" s="2"/>
+      <c r="H961" s="2"/>
+      <c r="I961" s="2"/>
+      <c r="J961" s="2"/>
+      <c r="K961" s="2"/>
+      <c r="L961" s="2"/>
+      <c r="M961" s="2"/>
+      <c r="N961" s="2"/>
+      <c r="O961" s="2"/>
+      <c r="P961" s="2"/>
+      <c r="Q961" s="2"/>
+      <c r="R961" s="2"/>
+      <c r="S961" s="2"/>
+      <c r="T961" s="2"/>
+      <c r="U961" s="2"/>
+      <c r="V961" s="2"/>
+      <c r="W961" s="2"/>
+      <c r="X961" s="2"/>
+      <c r="Y961" s="2"/>
+      <c r="Z961" s="2"/>
+    </row>
+    <row r="962" ht="15.75" customHeight="1">
+      <c r="A962" s="2"/>
+      <c r="B962" s="2"/>
+      <c r="C962" s="2"/>
+      <c r="D962" s="2"/>
+      <c r="E962" s="2"/>
+      <c r="F962" s="2"/>
+      <c r="G962" s="2"/>
+      <c r="H962" s="2"/>
+      <c r="I962" s="2"/>
+      <c r="J962" s="2"/>
+      <c r="K962" s="2"/>
+      <c r="L962" s="2"/>
+      <c r="M962" s="2"/>
+      <c r="N962" s="2"/>
+      <c r="O962" s="2"/>
+      <c r="P962" s="2"/>
+      <c r="Q962" s="2"/>
+      <c r="R962" s="2"/>
+      <c r="S962" s="2"/>
+      <c r="T962" s="2"/>
+      <c r="U962" s="2"/>
+      <c r="V962" s="2"/>
+      <c r="W962" s="2"/>
+      <c r="X962" s="2"/>
+      <c r="Y962" s="2"/>
+      <c r="Z962" s="2"/>
+    </row>
+    <row r="963" ht="15.75" customHeight="1">
+      <c r="A963" s="2"/>
+      <c r="B963" s="2"/>
+      <c r="C963" s="2"/>
+      <c r="D963" s="2"/>
+      <c r="E963" s="2"/>
+      <c r="F963" s="2"/>
+      <c r="G963" s="2"/>
+      <c r="H963" s="2"/>
+      <c r="I963" s="2"/>
+      <c r="J963" s="2"/>
+      <c r="K963" s="2"/>
+      <c r="L963" s="2"/>
+      <c r="M963" s="2"/>
+      <c r="N963" s="2"/>
+      <c r="O963" s="2"/>
+      <c r="P963" s="2"/>
+      <c r="Q963" s="2"/>
+      <c r="R963" s="2"/>
+      <c r="S963" s="2"/>
+      <c r="T963" s="2"/>
+      <c r="U963" s="2"/>
+      <c r="V963" s="2"/>
+      <c r="W963" s="2"/>
+      <c r="X963" s="2"/>
+      <c r="Y963" s="2"/>
+      <c r="Z963" s="2"/>
+    </row>
+    <row r="964" ht="15.75" customHeight="1">
+      <c r="A964" s="2"/>
+      <c r="B964" s="2"/>
+      <c r="C964" s="2"/>
+      <c r="D964" s="2"/>
+      <c r="E964" s="2"/>
+      <c r="F964" s="2"/>
+      <c r="G964" s="2"/>
+      <c r="H964" s="2"/>
+      <c r="I964" s="2"/>
+      <c r="J964" s="2"/>
+      <c r="K964" s="2"/>
+      <c r="L964" s="2"/>
+      <c r="M964" s="2"/>
+      <c r="N964" s="2"/>
+      <c r="O964" s="2"/>
+      <c r="P964" s="2"/>
+      <c r="Q964" s="2"/>
+      <c r="R964" s="2"/>
+      <c r="S964" s="2"/>
+      <c r="T964" s="2"/>
+      <c r="U964" s="2"/>
+      <c r="V964" s="2"/>
+      <c r="W964" s="2"/>
+      <c r="X964" s="2"/>
+      <c r="Y964" s="2"/>
+      <c r="Z964" s="2"/>
+    </row>
+    <row r="965" ht="15.75" customHeight="1">
+      <c r="A965" s="2"/>
+      <c r="B965" s="2"/>
+      <c r="C965" s="2"/>
+      <c r="D965" s="2"/>
+      <c r="E965" s="2"/>
+      <c r="F965" s="2"/>
+      <c r="G965" s="2"/>
+      <c r="H965" s="2"/>
+      <c r="I965" s="2"/>
+      <c r="J965" s="2"/>
+      <c r="K965" s="2"/>
+      <c r="L965" s="2"/>
+      <c r="M965" s="2"/>
+      <c r="N965" s="2"/>
+      <c r="O965" s="2"/>
+      <c r="P965" s="2"/>
+      <c r="Q965" s="2"/>
+      <c r="R965" s="2"/>
+      <c r="S965" s="2"/>
+      <c r="T965" s="2"/>
+      <c r="U965" s="2"/>
+      <c r="V965" s="2"/>
+      <c r="W965" s="2"/>
+      <c r="X965" s="2"/>
+      <c r="Y965" s="2"/>
+      <c r="Z965" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A40:A42"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A47:H52"/>
+  <mergeCells count="16">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A16:H16"/>
@@ -28011,6 +28285,15 @@
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B29:F29"/>
+    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A53:H58"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="B51:F51"/>
   </mergeCells>
   <conditionalFormatting sqref="G29">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
@@ -28022,7 +28305,7 @@
   <pageSetup paperSize="9" orientation="landscape"/>
   <rowBreaks count="2" manualBreakCount="2">
     <brk man="1"/>
-    <brk id="52" man="1"/>
+    <brk id="58" man="1"/>
   </rowBreaks>
   <colBreaks count="2" manualBreakCount="2">
     <brk man="1"/>

</xml_diff>